<commit_message>
SCRUM-114: Run 1 — 9 кейсів, виконаних 28.10.2026 (TC-003, 005, 010, 012, 013, 023, 027, 029, 032): 7 failed, 2 passed, звіти #50–#58
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -664,6 +664,384 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>TC-003</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>#54</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Значення 100 замінено на 99; повідомлення «You can order at most 99 of this product.» — спливне вікно у правому верхньому куті, під полем «Quantity» немає (крок 3). Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>TC-005</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>#55</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Крок 3: поле «Password» без зірочки (решта обов'язкових — із зірочкою в підказці). Кроки 4–22 (реєстрація, вхід, вихід) не виконано. Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>TC-010</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>#57</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Крок 7: звернення прийнято, «Thanks for your message! We will contact you shortly.» показано замість форми, а не над нею. Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>TC-012</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>#53</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Крок 7: форму не надіслано, але помилка «The message field must not be greater than 250 characters.» — під кнопкою «Send», а не під полем «Message». Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>TC-013</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>#51</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Файл .png заблоковано, помилка біля поля «Attachment». Додатково поза кроками: непорожній .txt 1 КБ теж відхилено («File should be empty.») — звіт #51. Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>#58</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Порядок Price (Low - High) правильний на сторінках 1 і 2. Назви варіантів відрізняються від F-70 («Price (Low - High)», «CO₂ Rating (A - E)») — окремий звіт #58, за критерієм кейсу не failed. Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>TC-027</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>#52</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Крок 3: значення 0 мовчки замінено на 1, повідомлення про помилку немає. Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>TC-029</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>#56</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Крок 13: зображення на сторінці товару 640×432 (pliers01.avif, той самий файл, що на картці); картка 640×432 — ≥400, ок. Кроки 2–7 (час завантаження при 10 Мбіт/с) не виконано. Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>TC-032</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>#50</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Кроки 2–3: /account і /account/favorites → /auth/login, ок. Крок 13: після «Continue as Guest» і «Proceed to checkout» відкрито крок 3 «Billing Address» без входу. Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
SCRUM-114: Run 1 — TC-036 перевиконано після змін кейсу (curl, reviewed КТ 28.10.2026): failed, #59, крок 7 — HTTP/1.1 200 OK без Location; рядок blocked лишено
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Environment" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Run 1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1084,6 +1084,48 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>#59</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Повторне виконання після змін кейсу (curl, reviewed КТ 28.10.2026). Крок 1: адреса стала https://, каталог відкрито (перехід знову виконав браузер, redirectCount = 0). Крок 3: «Security» — з'єднання захищене, у «Connection» вказано QUIC, X25519MLKEM768, AES_128_GCM; назви «TLS 1.3» немає, але QUIC працює лише на TLS 1.3 (RFC 9001), curl до https:// — TLSv1.3. Крок 7: curl -sI http://practicesoftwaretesting.com/ → HTTP/1.1 200 OK без Location — сервер не перенаправляє HTTP на HTTPS, звіт #59. Вікно 1458×833 замість 1280×800 (Environment).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
SCRUM-114: Run 1 — ще 14 кейсів, виконаних 28.10.2026: 9 passed (TC-001, 009, 018, 020, 021, 022, 025, 033, 035), TC-011 failed (#57), 4 blocked (TC-002, 014, 024, 028: «Combination Pliers» Out of stock)
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1126,6 +1126,594 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>TC-001</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Результати під «Searched for: pliers»: 4 картки — Combination Pliers, Pliers, Long Nose Pliers, Slip Joint Pliers. Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>TC-002</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Передумову не виконано: «Combination Pliers» на demo «Out of stock», кнопка «Add to cart» неактивна (API: in_stock = false, перевірено двічі 28.10.2026 близько 20:20 і 20:40); кроки з кошиком виконати неможливо.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>TC-009</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Крок 7: форму не надіслано, під «Message» — «Message must be minimal 50 characters», під іншими полями помилок немає. Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>TC-011</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>#57</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Крок 7: звернення прийнято, але «Thanks for your message! We will contact you shortly.» показано замість форми, а не над нею — той самий дефект, що в TC-010 (#57), новий звіт не створено. Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>TC-014</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Передумову не виконано: «Combination Pliers» на demo «Out of stock», кнопка «Add to cart» неактивна (API: in_stock = false, перевірено двічі 28.10.2026 близько 20:20 і 20:40); кроки з кошиком виконати неможливо.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Крок 3: «Unauthorized, can not add product to your favorite list.», та сама сторінка товару, у меню «Sign in». Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>TC-020</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>9 карток, 3 ряди по 3; у кожній зображення, назва, CO2, ціна; навігація « 1 2 3 4 5 »; сторінка 2 — 9 інших карток; «Previous» повертає сторінку 1 (перша Combination Pliers, остання Thor Hammer). Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>TC-021</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Підкатегорії «Power Tools»: Grinder, Sander, Saw, Drill. Після прапорця без перезавантаження — 5 карток (Sheet Sander, Belt Sander, Circular Saw, Cordless Drill 24V, Cordless Drill 12V), без навігації; Sheet Sander — категорія Sander. Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>TC-022</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>«Searched for: Hammer», 6 карток, у кожній назві hammer; після «X» поле порожнє, 9 карток, перша Combination Pliers (як на кроці 2). Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Передумову не виконано: «Combination Pliers» на demo «Out of stock», кнопка «Add to cart» неактивна (API: in_stock = false, перевірено двічі 28.10.2026 близько 20:20 і 20:40); кроки з кошиком виконати неможливо.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>TC-025</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Крок 4: під полем «Email address» — «Email is required», адреса /auth/forgot-password не змінилася, повідомлення про надсилання немає. Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>TC-028</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Передумову не виконано: «Combination Pliers» на demo «Out of stock», кнопка «Add to cart» неактивна (API: in_stock = false, перевірено двічі 28.10.2026 близько 20:20 і 20:40); кроки з кошиком виконати неможливо.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>TC-033</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>«Searched for: xyzabc», карток немає, «There are no products found.»; після «X» — 9 карток і навігація. Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Мітки «Email address *», «Password *»; Tab: email → password → кнопка показу пароля → «Login»; Enter — «Email is required» і «Password is required» під полями, адреса /auth/login. Область сторінки 1280×793 замість 1280×800: висоту обмежує екран (Environment); нова сесія — очищено localStorage і sessionStorage.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
SCRUM-114: Run 1 — TC-030 passed: Lighthouse 12.6.1 Accessibility 0.96, контраст пройдено; шрифти 20/16/16 px і 16 px
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1672,6 +1672,48 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>TC-030</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, macOS 26.6.2</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Кроки 2–5: Lighthouse 12.6.1 (категорія Accessibility, Navigation, Desktop) запущено з термінала на тому самому рушії Chromium 156 у headless-режимі, а не з вкладки DevTools: оцінка Accessibility 0.96, аудит «Background and foreground colors have a sufficient contrast ratio» — у Passed audits. Крок 8: 20px, 16px, 16px; крок 11: 16px — усі не менше 14px. Поза критерієм кейсу Lighthouse не пройшли heading-order, label-content-name-mismatch, list. Область сторінки 1280×793 (Environment).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
SCRUM-114: Run 1 — TC-037 failed (виконала Коротка К., кроки 7–8: «File should be empty.»), #51
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1924,6 +1924,48 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>TC-037</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156, Windows 11</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>#51</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Кроки 1–6 — як очікувано. Кроки 7–8: після вибору note.txt (1 КБ) поле «Attachment» підсвічено червоним, «File should be empty.», форму не надіслано — той самий дефект, що #51, новий звіт не створено. Середовище — як у TC-031 за повідомленням виконавиці. Дані передала виконавиця, занесла Тимчак А.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
SCRUM-114: Run 1 — кейси Дрєпіної А.: TC-015, 016, 018, 025 passed; TC-017, 026 blocked (customer@ заблоковано)
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2134,6 +2134,258 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>TC-015</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156.0.8078.73, Windows 11 Pro 21H2</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Кроки 1–8 — як очікувано: вхід customer@, у меню «Jane Doe», /account. Вікно на весь екран, розмір не вимірювано (Environment). Дані передала виконавиця, занесла Тимчак А.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>TC-016</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156.0.8078.73, Windows 11 Pro 21H2</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Крок 5: «Invalid email or password», сеанс не створено. Вікно на весь екран, розмір не вимірювано (Environment). Дані передала виконавиця, занесла Тимчак А.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>TC-017</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156.0.8078.73, Windows 11 Pro 21H2</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Кроки 1–7 — як очікувано («Product added to shopping cart.» за ~1 с, кошик 1 × $14.15). Крок 8: Спільний обліковий запис customer@practicesoftwaretesting.com заблоковано: «Account locked, too many failed attempts. Please contact the administrator.» (пароль введено правильно; повторна перевірка 29.10.2026 08:53 — досі заблоковано). Середовище недоступне — blocked (п. 4.7). Вікно на весь екран, розмір не вимірювано (Environment). Дані передала виконавиця, занесла Тимчак А.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156.0.8078.73, Windows 11 Pro 21H2</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Крок 3: «Unauthorized, can not add product to your favorite list.», у меню «Sign in». Вікно на весь екран, розмір не вимірювано (Environment). Дані передала виконавиця, занесла Тимчак А.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>TC-025</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156.0.8078.73, Windows 11 Pro 21H2</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Крок 4: під полем «Email address» — «Email is required», адреса /auth/forgot-password не змінилася. Вікно на весь екран, розмір не вимірювано (Environment). Дані передала виконавиця, занесла Тимчак А.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>TC-026</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156.0.8078.73, Windows 11 Pro 21H2</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Крок 5: Спільний обліковий запис customer@practicesoftwaretesting.com заблоковано: «Account locked, too many failed attempts. Please contact the administrator.» (пароль введено правильно; повторна перевірка 29.10.2026 08:53 — досі заблоковано). Середовище недоступне — blocked (п. 4.7). Вікно на весь екран, розмір не вимірювано (Environment). Дані передала виконавиця, занесла Тимчак А.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
SCRUM-114: Run 1 — TC-019 failed (виконала Дрєпіна А., крок 19: «page.forgot-password.confirm»), #68
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -609,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2386,6 +2386,48 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>TC-019</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>збірка v2.5 від 2026-10-11; Chrome 156.0.8078.73, Windows 11 Pro 21H2</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>#68</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Крок 19: замість повідомлення про надсилання листа показано ключ локалізації «page.forgot-password.confirm», звіт #68. Адреса shopline.it.tc019.28102026b@example.com — повторний прогін: адреса з кейсу (без «b») уже була використана, тому додано «b». Вікно на весь екран, розмір не вимірювано (Environment). Дані передала виконавиця, занесла Тимчак А.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>